<commit_message>
AE-2081: adding openssl-3.6.2 and openssl-4.0.0
</commit_message>
<xml_diff>
--- a/tests/resources/workspace-001/crypto-bom-SNAPSHOT/02_prepared/crypto-bom-SNAPSHOT/crypto-bom-inventory.xlsx
+++ b/tests/resources/workspace-001/crypto-bom-SNAPSHOT/02_prepared/crypto-bom-SNAPSHOT/crypto-bom-inventory.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kklein/workspace/metaeffekt-workbench_gh/tests/resources/workspace-001/crypto-bom-SNAPSHOT/02_prepared/crypto-bom-SNAPSHOT/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC61A2E3-6D23-E94B-AD68-2D216525D27F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC39478D-D4C6-7F40-9178-5763B4D368DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="280" yWindow="980" windowWidth="22420" windowHeight="19660" xr2:uid="{C861F88B-F5CE-9A44-9AD9-8AB165D83E00}"/>
   </bookViews>
@@ -18,7 +18,7 @@
     <sheet name="Info" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">Artifacts!$A$1:$H$58</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">Artifacts!$A$1:$H$59</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1">Assets!$A$1:$C$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2">Info!$A$1:$C$2</definedName>
   </definedNames>
@@ -27,7 +27,9 @@
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
         <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
         <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
@@ -38,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="349" uniqueCount="201">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="356" uniqueCount="202">
   <si>
     <t>Id</t>
   </si>
@@ -112,15 +114,9 @@
     <t>Libgcrypt</t>
   </si>
   <si>
-    <t>openssl-3.6.1</t>
-  </si>
-  <si>
     <t>OpenSSL</t>
   </si>
   <si>
-    <t>3.6.1</t>
-  </si>
-  <si>
     <t>gnutls-3.8.12</t>
   </si>
   <si>
@@ -641,6 +637,15 @@
   </si>
   <si>
     <t>pkg:rpm/redhat/libsodium</t>
+  </si>
+  <si>
+    <t>openssl-3.6.2</t>
+  </si>
+  <si>
+    <t>3.6.2</t>
+  </si>
+  <si>
+    <t>openssl-4.0.0</t>
   </si>
 </sst>
 </file>
@@ -1112,7 +1117,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D27CFD85-162E-2944-8AF0-B3BE97F22723}">
-  <dimension ref="A1:H58"/>
+  <dimension ref="A1:H59"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="20.83203125" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="21" bestFit="1" customWidth="1"/>
@@ -1142,24 +1147,24 @@
         <v>2</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A2" t="s">
+        <v>155</v>
+      </c>
+      <c r="B2" t="s">
+        <v>156</v>
+      </c>
+      <c r="C2" t="s">
         <v>157</v>
-      </c>
-      <c r="B2" t="s">
-        <v>158</v>
-      </c>
-      <c r="C2" t="s">
-        <v>159</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>4</v>
@@ -1170,13 +1175,13 @@
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A3" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="C3" s="4" t="s">
         <v>58</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>60</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>4</v>
@@ -1186,19 +1191,19 @@
       </c>
       <c r="F3" s="3"/>
       <c r="G3" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A4" s="3" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="B4" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="C4" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="C4" s="4" t="s">
-        <v>53</v>
-      </c>
       <c r="D4" s="2" t="s">
         <v>4</v>
       </c>
@@ -1206,10 +1211,10 @@
         <v>5</v>
       </c>
       <c r="F4" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="H4" s="3"/>
     </row>
@@ -1218,7 +1223,7 @@
         <v>18</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>19</v>
@@ -1230,22 +1235,22 @@
         <v>5</v>
       </c>
       <c r="F5" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="H5" s="3"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A6" s="3" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>4</v>
@@ -1259,13 +1264,13 @@
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A7" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="B7" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="B7" s="3" t="s">
-        <v>47</v>
-      </c>
       <c r="C7" s="4" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>4</v>
@@ -1279,13 +1284,13 @@
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A8" s="3" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>4</v>
@@ -1297,13 +1302,13 @@
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A9" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="C9" s="4" t="s">
         <v>61</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>63</v>
       </c>
       <c r="D9" s="2" t="s">
         <v>4</v>
@@ -1330,18 +1335,18 @@
         <v>5</v>
       </c>
       <c r="G10" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A11" s="3" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B11" s="3" t="s">
         <v>12</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="D11" s="2" t="s">
         <v>4</v>
@@ -1350,18 +1355,18 @@
         <v>5</v>
       </c>
       <c r="G11" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A12" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="B12" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="B12" s="3" t="s">
-        <v>66</v>
-      </c>
       <c r="C12" s="4" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="D12" s="2" t="s">
         <v>4</v>
@@ -1370,22 +1375,22 @@
         <v>5</v>
       </c>
       <c r="F12" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="G12" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A13" t="s">
+        <v>160</v>
+      </c>
+      <c r="B13" t="s">
+        <v>161</v>
+      </c>
+      <c r="C13" t="s">
         <v>162</v>
       </c>
-      <c r="B13" t="s">
-        <v>163</v>
-      </c>
-      <c r="C13" t="s">
-        <v>164</v>
-      </c>
       <c r="D13" s="2" t="s">
         <v>4</v>
       </c>
@@ -1393,18 +1398,18 @@
         <v>5</v>
       </c>
       <c r="F13" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A14" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="C14" s="4" t="s">
         <v>67</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="C14" s="4" t="s">
-        <v>69</v>
       </c>
       <c r="D14" s="2" t="s">
         <v>4</v>
@@ -1414,18 +1419,18 @@
       </c>
       <c r="F14" s="3"/>
       <c r="G14" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A15" s="3" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="D15" s="2" t="s">
         <v>4</v>
@@ -1437,13 +1442,13 @@
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A16" s="3" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="D16" s="2" t="s">
         <v>4</v>
@@ -1455,13 +1460,13 @@
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A17" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="C17" s="4" t="s">
         <v>73</v>
-      </c>
-      <c r="B17" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="C17" s="4" t="s">
-        <v>75</v>
       </c>
       <c r="D17" s="2" t="s">
         <v>4</v>
@@ -1473,13 +1478,13 @@
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A18" s="3" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="D18" s="2" t="s">
         <v>4</v>
@@ -1489,18 +1494,18 @@
       </c>
       <c r="F18" s="3"/>
       <c r="G18" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A19" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="C19" s="4" t="s">
         <v>27</v>
-      </c>
-      <c r="B19" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="C19" s="4" t="s">
-        <v>29</v>
       </c>
       <c r="D19" s="2" t="s">
         <v>4</v>
@@ -1510,18 +1515,18 @@
       </c>
       <c r="F19" s="3"/>
       <c r="G19" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A20" s="3" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="D20" s="2" t="s">
         <v>4</v>
@@ -1530,21 +1535,21 @@
         <v>5</v>
       </c>
       <c r="F20" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="G20" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A21" s="3" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="D21" s="2" t="s">
         <v>4</v>
@@ -1553,10 +1558,10 @@
         <v>5</v>
       </c>
       <c r="F21" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="G21" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.15">
@@ -1581,14 +1586,14 @@
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A23" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="C23" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="B23" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="C23" s="4" t="s">
-        <v>79</v>
-      </c>
       <c r="D23" s="2" t="s">
         <v>4</v>
       </c>
@@ -1596,21 +1601,21 @@
         <v>5</v>
       </c>
       <c r="F23" s="3" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="H23" s="6" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A24" s="3" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B24" s="3" t="s">
         <v>23</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="D24" s="2" t="s">
         <v>4</v>
@@ -1620,18 +1625,18 @@
       </c>
       <c r="F24" s="3"/>
       <c r="G24" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A25" s="3" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B25" s="3" t="s">
         <v>23</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D25" s="2" t="s">
         <v>4</v>
@@ -1641,18 +1646,18 @@
       </c>
       <c r="F25" s="3"/>
       <c r="G25" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A26" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="B26" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="C26" s="4" t="s">
         <v>91</v>
-      </c>
-      <c r="B26" s="3" t="s">
-        <v>92</v>
-      </c>
-      <c r="C26" s="4" t="s">
-        <v>93</v>
       </c>
       <c r="D26" s="2" t="s">
         <v>4</v>
@@ -1662,18 +1667,18 @@
       </c>
       <c r="F26" s="3"/>
       <c r="G26" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A27" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="B27" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="C27" s="4" t="s">
         <v>95</v>
-      </c>
-      <c r="B27" s="3" t="s">
-        <v>96</v>
-      </c>
-      <c r="C27" s="4" t="s">
-        <v>97</v>
       </c>
       <c r="D27" s="2" t="s">
         <v>4</v>
@@ -1685,13 +1690,13 @@
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A28" s="3" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="D28" s="2" t="s">
         <v>4</v>
@@ -1700,19 +1705,19 @@
         <v>5</v>
       </c>
       <c r="H28" s="6" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A29" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="B29" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="C29" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="B29" s="3" t="s">
-        <v>99</v>
-      </c>
-      <c r="C29" s="4" t="s">
-        <v>100</v>
-      </c>
       <c r="D29" s="2" t="s">
         <v>4</v>
       </c>
@@ -1720,18 +1725,18 @@
         <v>5</v>
       </c>
       <c r="H29" s="6" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A30" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="B30" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="C30" s="4" t="s">
         <v>103</v>
-      </c>
-      <c r="B30" s="3" t="s">
-        <v>104</v>
-      </c>
-      <c r="C30" s="4" t="s">
-        <v>105</v>
       </c>
       <c r="D30" s="2" t="s">
         <v>4</v>
@@ -1741,18 +1746,18 @@
       </c>
       <c r="F30" s="3"/>
       <c r="G30" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A31" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="B31" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="C31" s="4" t="s">
         <v>106</v>
-      </c>
-      <c r="B31" s="3" t="s">
-        <v>107</v>
-      </c>
-      <c r="C31" s="4" t="s">
-        <v>108</v>
       </c>
       <c r="D31" s="2" t="s">
         <v>4</v>
@@ -1762,18 +1767,18 @@
       </c>
       <c r="F31" s="3"/>
       <c r="G31" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A32" s="3" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="D32" s="2" t="s">
         <v>4</v>
@@ -1785,13 +1790,13 @@
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.15">
       <c r="A33" s="3" t="s">
+        <v>171</v>
+      </c>
+      <c r="B33" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="C33" s="4" t="s">
         <v>173</v>
-      </c>
-      <c r="B33" s="3" t="s">
-        <v>174</v>
-      </c>
-      <c r="C33" s="4" t="s">
-        <v>175</v>
       </c>
       <c r="D33" s="2" t="s">
         <v>4</v>
@@ -1803,13 +1808,13 @@
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.15">
       <c r="A34" s="3" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="D34" s="2" t="s">
         <v>4</v>
@@ -1821,13 +1826,13 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.15">
       <c r="A35" s="3" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="B35" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="C35" s="4" t="s">
         <v>109</v>
-      </c>
-      <c r="C35" s="4" t="s">
-        <v>111</v>
       </c>
       <c r="D35" s="2" t="s">
         <v>4</v>
@@ -1839,13 +1844,13 @@
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.15">
       <c r="A36" s="3" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="D36" s="2" t="s">
         <v>4</v>
@@ -1857,13 +1862,13 @@
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.15">
       <c r="A37" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="B37" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="C37" s="4" t="s">
         <v>112</v>
-      </c>
-      <c r="B37" s="3" t="s">
-        <v>113</v>
-      </c>
-      <c r="C37" s="4" t="s">
-        <v>114</v>
       </c>
       <c r="D37" s="2" t="s">
         <v>4</v>
@@ -1873,19 +1878,19 @@
       </c>
       <c r="F37" s="3"/>
       <c r="G37" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.15">
       <c r="A38" s="3" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="B38" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="C38" s="4" t="s">
         <v>115</v>
       </c>
-      <c r="C38" s="4" t="s">
-        <v>117</v>
-      </c>
       <c r="D38" s="2" t="s">
         <v>4</v>
       </c>
@@ -1893,21 +1898,21 @@
         <v>5</v>
       </c>
       <c r="F38" s="3" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="G38" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.15">
       <c r="A39" s="3" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="B39" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="C39" s="4" t="s">
         <v>118</v>
-      </c>
-      <c r="C39" s="4" t="s">
-        <v>120</v>
       </c>
       <c r="D39" s="2" t="s">
         <v>4</v>
@@ -1919,13 +1924,13 @@
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.15">
       <c r="A40" s="3" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="D40" s="2" t="s">
         <v>4</v>
@@ -1934,19 +1939,19 @@
         <v>5</v>
       </c>
       <c r="G40" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.15">
       <c r="A41" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="B41" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="C41" s="4" t="s">
         <v>124</v>
       </c>
-      <c r="B41" s="3" t="s">
-        <v>125</v>
-      </c>
-      <c r="C41" s="4" t="s">
-        <v>126</v>
-      </c>
       <c r="D41" s="2" t="s">
         <v>4</v>
       </c>
@@ -1954,18 +1959,18 @@
         <v>5</v>
       </c>
       <c r="G41" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.15">
       <c r="A42" s="3" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="D42" s="2" t="s">
         <v>4</v>
@@ -1977,13 +1982,13 @@
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.15">
       <c r="A43" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="B43" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="B43" s="3" t="s">
-        <v>57</v>
-      </c>
       <c r="C43" s="3" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="D43" s="2" t="s">
         <v>4</v>
@@ -1995,13 +2000,13 @@
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.15">
       <c r="A44" s="3" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B44" s="3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C44" s="4" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="D44" s="2" t="s">
         <v>4</v>
@@ -2010,21 +2015,21 @@
         <v>5</v>
       </c>
       <c r="F44" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="G44" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.15">
       <c r="A45" s="3" t="s">
+        <v>199</v>
+      </c>
+      <c r="B45" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="B45" s="3" t="s">
-        <v>25</v>
-      </c>
       <c r="C45" s="4" t="s">
-        <v>26</v>
+        <v>200</v>
       </c>
       <c r="D45" s="2" t="s">
         <v>4</v>
@@ -2033,112 +2038,118 @@
         <v>5</v>
       </c>
       <c r="F45" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="G45" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.15">
       <c r="A46" s="3" t="s">
-        <v>129</v>
-      </c>
-      <c r="B46" t="s">
-        <v>130</v>
+        <v>201</v>
+      </c>
+      <c r="B46" s="3" t="s">
+        <v>24</v>
       </c>
       <c r="C46" s="4" t="s">
-        <v>131</v>
+        <v>112</v>
       </c>
       <c r="D46" s="2" t="s">
         <v>4</v>
       </c>
       <c r="E46" s="3" t="s">
         <v>5</v>
+      </c>
+      <c r="F46" t="s">
+        <v>195</v>
+      </c>
+      <c r="G46" t="s">
+        <v>181</v>
       </c>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.15">
       <c r="A47" s="3" t="s">
-        <v>138</v>
-      </c>
-      <c r="B47" s="3" t="s">
-        <v>133</v>
-      </c>
-      <c r="C47" s="3" t="s">
-        <v>139</v>
+        <v>127</v>
+      </c>
+      <c r="B47" t="s">
+        <v>128</v>
+      </c>
+      <c r="C47" s="4" t="s">
+        <v>129</v>
       </c>
       <c r="D47" s="2" t="s">
         <v>4</v>
       </c>
       <c r="E47" s="3" t="s">
-        <v>142</v>
-      </c>
-      <c r="G47" t="s">
-        <v>184</v>
+        <v>5</v>
       </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.15">
       <c r="A48" s="3" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="B48" s="3" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="C48" s="3" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="D48" s="2" t="s">
         <v>4</v>
       </c>
       <c r="E48" s="3" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="G48" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.15">
       <c r="A49" s="3" t="s">
-        <v>135</v>
-      </c>
-      <c r="B49" t="s">
-        <v>136</v>
+        <v>130</v>
+      </c>
+      <c r="B49" s="3" t="s">
+        <v>131</v>
       </c>
       <c r="C49" s="3" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="D49" s="2" t="s">
         <v>4</v>
       </c>
       <c r="E49" s="3" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="G49" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.15">
       <c r="A50" s="3" t="s">
-        <v>144</v>
+        <v>133</v>
       </c>
       <c r="B50" t="s">
+        <v>134</v>
+      </c>
+      <c r="C50" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="D50" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="E50" s="3" t="s">
         <v>140</v>
       </c>
-      <c r="C50" s="4" t="s">
-        <v>145</v>
-      </c>
-      <c r="D50" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="E50" s="3" t="s">
-        <v>142</v>
+      <c r="G50" t="s">
+        <v>183</v>
       </c>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.15">
       <c r="A51" s="3" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="B51" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="C51" s="4" t="s">
         <v>143</v>
@@ -2147,72 +2158,69 @@
         <v>4</v>
       </c>
       <c r="E51" s="3" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.15">
       <c r="A52" s="3" t="s">
-        <v>147</v>
-      </c>
-      <c r="B52" s="3" t="s">
-        <v>146</v>
+        <v>139</v>
+      </c>
+      <c r="B52" t="s">
+        <v>138</v>
       </c>
       <c r="C52" s="4" t="s">
-        <v>148</v>
+        <v>141</v>
       </c>
       <c r="D52" s="2" t="s">
         <v>4</v>
       </c>
       <c r="E52" s="3" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.15">
       <c r="A53" s="3" t="s">
-        <v>186</v>
+        <v>145</v>
       </c>
       <c r="B53" s="3" t="s">
-        <v>187</v>
+        <v>144</v>
       </c>
       <c r="C53" s="4" t="s">
-        <v>111</v>
+        <v>146</v>
       </c>
       <c r="D53" s="2" t="s">
         <v>4</v>
       </c>
       <c r="E53" s="3" t="s">
-        <v>5</v>
+        <v>140</v>
       </c>
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.15">
       <c r="A54" s="3" t="s">
-        <v>150</v>
+        <v>184</v>
       </c>
       <c r="B54" s="3" t="s">
-        <v>149</v>
+        <v>185</v>
       </c>
       <c r="C54" s="4" t="s">
-        <v>151</v>
+        <v>109</v>
       </c>
       <c r="D54" s="2" t="s">
         <v>4</v>
       </c>
       <c r="E54" s="3" t="s">
         <v>5</v>
-      </c>
-      <c r="G54" t="s">
-        <v>188</v>
       </c>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.15">
       <c r="A55" s="3" t="s">
-        <v>153</v>
+        <v>148</v>
       </c>
       <c r="B55" s="3" t="s">
-        <v>152</v>
+        <v>147</v>
       </c>
       <c r="C55" s="4" t="s">
-        <v>154</v>
+        <v>149</v>
       </c>
       <c r="D55" s="2" t="s">
         <v>4</v>
@@ -2221,18 +2229,18 @@
         <v>5</v>
       </c>
       <c r="G55" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.15">
       <c r="A56" s="3" t="s">
-        <v>43</v>
+        <v>151</v>
       </c>
       <c r="B56" s="3" t="s">
-        <v>41</v>
+        <v>150</v>
       </c>
       <c r="C56" s="4" t="s">
-        <v>44</v>
+        <v>152</v>
       </c>
       <c r="D56" s="2" t="s">
         <v>4</v>
@@ -2240,19 +2248,16 @@
       <c r="E56" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="F56" t="s">
-        <v>198</v>
-      </c>
       <c r="G56" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.15">
       <c r="A57" s="3" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B57" s="3" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C57" s="4" t="s">
         <v>42</v>
@@ -2264,21 +2269,21 @@
         <v>5</v>
       </c>
       <c r="F57" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="G57" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.15">
       <c r="A58" s="3" t="s">
-        <v>155</v>
+        <v>38</v>
       </c>
       <c r="B58" s="3" t="s">
-        <v>156</v>
+        <v>39</v>
       </c>
       <c r="C58" s="4" t="s">
-        <v>111</v>
+        <v>40</v>
       </c>
       <c r="D58" s="2" t="s">
         <v>4</v>
@@ -2286,9 +2291,32 @@
       <c r="E58" s="3" t="s">
         <v>5</v>
       </c>
+      <c r="F58" t="s">
+        <v>196</v>
+      </c>
+      <c r="G58" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7" x14ac:dyDescent="0.15">
+      <c r="A59" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="B59" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="C59" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="D59" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="E59" s="3" t="s">
+        <v>5</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H58" xr:uid="{D27CFD85-162E-2944-8AF0-B3BE97F22723}"/>
+  <autoFilter ref="A1:H59" xr:uid="{D27CFD85-162E-2944-8AF0-B3BE97F22723}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
   <headerFooter alignWithMargins="0"/>

</xml_diff>

<commit_message>
fixed license reports for sample-product
</commit_message>
<xml_diff>
--- a/tests/resources/workspace-001/crypto-bom-SNAPSHOT/02_prepared/crypto-bom-SNAPSHOT/crypto-bom-inventory.xlsx
+++ b/tests/resources/workspace-001/crypto-bom-SNAPSHOT/02_prepared/crypto-bom-SNAPSHOT/crypto-bom-inventory.xlsx
@@ -24,6 +24,21 @@
     <t>Id</t>
   </si>
   <si>
+    <t>Footer</t>
+  </si>
+  <si>
+    <t>Title</t>
+  </si>
+  <si>
+    <t>vad-customization</t>
+  </si>
+  <si>
+    <t>CryptoBOM SNAPSHOT</t>
+  </si>
+  <si>
+    <t>CryptoBOM SNAPSHOT Assessment</t>
+  </si>
+  <si>
     <t>Component</t>
   </si>
   <si>
@@ -601,21 +616,6 @@
   </si>
   <si>
     <t>yescrypt</t>
-  </si>
-  <si>
-    <t>Footer</t>
-  </si>
-  <si>
-    <t>Title</t>
-  </si>
-  <si>
-    <t>vad-customization</t>
-  </si>
-  <si>
-    <t>CryptoBOM SNAPSHOT</t>
-  </si>
-  <si>
-    <t>CryptoBOM SNAPSHOT Assessment</t>
   </si>
   <si>
     <t>Asset Id</t>
@@ -842,1149 +842,1149 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="B2" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="C2" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="D2" s="9" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="E2" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="B3" t="s">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="C3" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="D3" s="9" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="E3" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="G3" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="B4" t="s">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="C4" t="s">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="E4" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="F4" t="s">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="G4" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="B5" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="C5" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="E5" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="F5" t="s">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="G5" t="s">
-        <v>25</v>
+        <v>30</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="B6" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="C6" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="E6" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="B7" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="C7" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="E7" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="B8" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="C8" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="E8" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="B9" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="C9" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="E9" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="B10" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="C10" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="E10" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="G10" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="B11" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="C11" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="D11" s="9" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="E11" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="G11" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="B12" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="C12" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="E12" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="F12" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="G12" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="B13" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="C13" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="D13" s="9" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="E13" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="F13" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="B14" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="C14" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="D14" s="9" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="E14" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="G14" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="B15" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="C15" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="D15" s="9" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="E15" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="B16" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="C16" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="D16" s="9" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="E16" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="B17" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="C17" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="D17" s="9" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="E17" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="B18" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="C18" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="E18" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="G18" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="B19" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="C19" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="D19" s="9" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="E19" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="G19" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="B20" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="C20" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="D20" s="9" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="E20" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="F20" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="G20" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="B21" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="C21" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="D21" s="9" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="E21" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="F21" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="G21" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="B22" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="C22" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="D22" s="9" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="E22" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="B23" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="C23" t="s">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="D23" s="9" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="E23" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="F23" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="H23" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="B24" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="C24" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="D24" s="9" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="E24" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="G24" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="B25" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="C25" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="D25" s="9" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="E25" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="G25" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="B26" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="C26" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="D26" s="9" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="E26" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="G26" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="B27" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="C27" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="D27" s="9" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="E27" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="B28" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="C28" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="D28" s="9" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="E28" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="H28" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="B29" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="C29" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="D29" s="9" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="E29" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="H29" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="B30" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="C30" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="D30" s="9" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="E30" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="G30" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="B31" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="C31" t="s">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="D31" s="9" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="E31" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="G31" t="s">
-        <v>110</v>
+        <v>115</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="B32" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="C32" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="D32" s="9" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="E32" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="B33" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="C33" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
       <c r="D33" s="9" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="E33" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="B34" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="C34" t="s">
-        <v>118</v>
+        <v>123</v>
       </c>
       <c r="D34" s="9" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="E34" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="B35" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="C35" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="D35" s="9" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="E35" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="B36" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="C36" t="s">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="D36" s="9" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="E36" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B37" t="s">
-        <v>124</v>
+        <v>129</v>
       </c>
       <c r="C37" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="D37" s="9" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="E37" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="G37" t="s">
-        <v>126</v>
+        <v>131</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="s">
-        <v>127</v>
+        <v>132</v>
       </c>
       <c r="B38" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="C38" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
       <c r="D38" s="9" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="E38" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="F38" t="s">
-        <v>130</v>
+        <v>135</v>
       </c>
       <c r="G38" t="s">
-        <v>131</v>
+        <v>136</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="B39" t="s">
-        <v>133</v>
+        <v>138</v>
       </c>
       <c r="C39" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="D39" s="9" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="E39" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="B40" t="s">
-        <v>136</v>
+        <v>141</v>
       </c>
       <c r="C40" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="D40" s="9" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="E40" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="G40" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
       <c r="B41" t="s">
-        <v>136</v>
+        <v>141</v>
       </c>
       <c r="C41" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
       <c r="D41" s="9" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="E41" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="G41" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
       <c r="B42" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="C42" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="D42" s="9" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="E42" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
       <c r="B43" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="C43" t="s">
-        <v>145</v>
+        <v>150</v>
       </c>
       <c r="D43" s="9" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="E43" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="s">
-        <v>146</v>
+        <v>151</v>
       </c>
       <c r="B44" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="C44" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="D44" s="9" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="E44" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="F44" t="s">
-        <v>149</v>
+        <v>154</v>
       </c>
       <c r="G44" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="B45" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="C45" t="s">
-        <v>152</v>
+        <v>157</v>
       </c>
       <c r="D45" s="9" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="E45" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="F45" t="s">
-        <v>149</v>
+        <v>154</v>
       </c>
       <c r="G45" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="s">
-        <v>153</v>
+        <v>158</v>
       </c>
       <c r="B46" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="C46" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="D46" s="9" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="E46" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="F46" t="s">
-        <v>149</v>
+        <v>154</v>
       </c>
       <c r="G46" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
       <c r="B47" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="C47" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="D47" s="9" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="E47" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="s">
-        <v>157</v>
+        <v>162</v>
       </c>
       <c r="B48" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="C48" t="s">
-        <v>159</v>
+        <v>164</v>
       </c>
       <c r="D48" s="9" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="E48" t="s">
-        <v>160</v>
+        <v>165</v>
       </c>
       <c r="G48" t="s">
-        <v>161</v>
+        <v>166</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
       <c r="B49" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="C49" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="D49" s="9" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="E49" t="s">
-        <v>160</v>
+        <v>165</v>
       </c>
       <c r="G49" t="s">
-        <v>161</v>
+        <v>166</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="s">
-        <v>164</v>
+        <v>169</v>
       </c>
       <c r="B50" t="s">
+        <v>170</v>
+      </c>
+      <c r="C50" t="s">
+        <v>171</v>
+      </c>
+      <c r="D50" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="E50" t="s">
         <v>165</v>
       </c>
-      <c r="C50" t="s">
-        <v>166</v>
-      </c>
-      <c r="D50" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="E50" t="s">
-        <v>160</v>
-      </c>
       <c r="G50" t="s">
-        <v>167</v>
+        <v>172</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="s">
-        <v>168</v>
+        <v>173</v>
       </c>
       <c r="B51" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
       <c r="C51" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="D51" s="9" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="E51" t="s">
-        <v>160</v>
+        <v>165</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="s">
-        <v>171</v>
+        <v>176</v>
       </c>
       <c r="B52" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
       <c r="C52" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="D52" s="9" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="E52" t="s">
-        <v>160</v>
+        <v>165</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="s">
-        <v>173</v>
+        <v>178</v>
       </c>
       <c r="B53" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="C53" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="D53" s="9" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="E53" t="s">
-        <v>160</v>
+        <v>165</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="B54" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="C54" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="D54" s="9" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="E54" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="B55" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="C55" t="s">
-        <v>180</v>
+        <v>185</v>
       </c>
       <c r="D55" s="9" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="E55" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="G55" t="s">
-        <v>181</v>
+        <v>186</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="s">
-        <v>182</v>
+        <v>187</v>
       </c>
       <c r="B56" t="s">
-        <v>183</v>
+        <v>188</v>
       </c>
       <c r="C56" t="s">
-        <v>184</v>
+        <v>189</v>
       </c>
       <c r="D56" s="9" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="E56" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="G56" t="s">
-        <v>181</v>
+        <v>186</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="s">
-        <v>185</v>
+        <v>190</v>
       </c>
       <c r="B57" t="s">
-        <v>186</v>
+        <v>191</v>
       </c>
       <c r="C57" t="s">
-        <v>187</v>
+        <v>192</v>
       </c>
       <c r="D57" s="9" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="E57" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="F57" t="s">
-        <v>188</v>
+        <v>193</v>
       </c>
       <c r="G57" t="s">
-        <v>189</v>
+        <v>194</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="s">
-        <v>190</v>
+        <v>195</v>
       </c>
       <c r="B58" t="s">
-        <v>186</v>
+        <v>191</v>
       </c>
       <c r="C58" t="s">
-        <v>191</v>
+        <v>196</v>
       </c>
       <c r="D58" s="9" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="E58" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="F58" t="s">
-        <v>188</v>
+        <v>193</v>
       </c>
       <c r="G58" t="s">
-        <v>189</v>
+        <v>194</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="s">
-        <v>192</v>
+        <v>197</v>
       </c>
       <c r="B59" t="s">
-        <v>193</v>
+        <v>198</v>
       </c>
       <c r="C59" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="D59" s="9" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="E59" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
     </row>
   </sheetData>
@@ -2006,12 +2006,12 @@
         <v>200</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>2</v>
+        <v>7</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="B2" t="s">
         <v>201</v>
@@ -2036,21 +2036,21 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>194</v>
+        <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>195</v>
+        <v>2</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>196</v>
+        <v>3</v>
       </c>
       <c r="B2" t="s">
-        <v>197</v>
+        <v>4</v>
       </c>
       <c r="C2" t="s">
-        <v>198</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>